<commit_message>
Updated the models with extra info
</commit_message>
<xml_diff>
--- a/QCOM.xlsx
+++ b/QCOM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/KINGSTON/MyStockData/Finance-StockLists/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7D40E9A-F16E-AD4B-A534-7C36DE678E6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2840191-F312-1547-A563-46C45B48FD7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="14400" xr2:uid="{AEC0C047-6E16-294C-82BD-58123BA913A1}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="14400" firstSheet="5" activeTab="14" xr2:uid="{AEC0C047-6E16-294C-82BD-58123BA913A1}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="2" r:id="rId1"/>
@@ -7312,17 +7312,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="E17:I17"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="C39:L39"/>
     <mergeCell ref="C3:G3"/>
     <mergeCell ref="H3:L3"/>
     <mergeCell ref="P3:W3"/>
     <mergeCell ref="X3:Z3"/>
     <mergeCell ref="C5:L5"/>
     <mergeCell ref="P5:Z5"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="E17:I17"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="C39:L39"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -33472,12 +33472,6 @@
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="C3:G3"/>
-    <mergeCell ref="H3:L3"/>
-    <mergeCell ref="P3:W3"/>
-    <mergeCell ref="X3:Z3"/>
-    <mergeCell ref="C5:L5"/>
-    <mergeCell ref="P5:Z5"/>
     <mergeCell ref="C40:L40"/>
     <mergeCell ref="C11:L11"/>
     <mergeCell ref="P11:Z11"/>
@@ -33485,6 +33479,12 @@
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="C26:L26"/>
     <mergeCell ref="C33:L33"/>
+    <mergeCell ref="C3:G3"/>
+    <mergeCell ref="H3:L3"/>
+    <mergeCell ref="P3:W3"/>
+    <mergeCell ref="X3:Z3"/>
+    <mergeCell ref="C5:L5"/>
+    <mergeCell ref="P5:Z5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>

</xml_diff>